<commit_message>
Combine Product/Technical Head role and remove Release Manager role title
- Ownership now: Product Owner: Sridhar Muppidi; Product / Technical Head:
  Sachin Tulla; Head of Engineering: Hari PS; Security Head: Anil M.
- Replace the "Release Manager" role title with "Head of Engineering" across docs
  (kept the technical term "secrets manager").
- Applied to Docs 01-04, 07-10 (Markdown + Word) and spreadsheets 05/06/07.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/compliance/07-SDLC-Change-Management-Tracker.xlsx
+++ b/docs/compliance/07-SDLC-Change-Management-Tracker.xlsx
@@ -559,7 +559,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Document ownership — Product Owner: Sridhar Muppidi | Product Head: Sachin Tulla | Technical Head: Sachin Tulla | Head of Engineering: Hari PS | Security Head: Anil M</t>
+          <t>Document ownership — Product Owner: Sridhar Muppidi | Product / Technical Head: Sachin Tulla | Head of Engineering: Hari PS | Security Head: Anil M</t>
         </is>
       </c>
     </row>
@@ -712,7 +712,7 @@
       </c>
       <c r="K2" s="3" t="inlineStr">
         <is>
-          <t>Release mgr</t>
+          <t>Head of Engineering</t>
         </is>
       </c>
       <c r="L2" s="3" t="inlineStr">
@@ -779,7 +779,7 @@
       </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>Release mgr</t>
+          <t>Head of Engineering</t>
         </is>
       </c>
       <c r="L3" s="3" t="inlineStr">
@@ -846,7 +846,7 @@
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>Release mgr</t>
+          <t>Head of Engineering</t>
         </is>
       </c>
       <c r="L4" s="3" t="inlineStr">
@@ -913,7 +913,7 @@
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t>Release mgr</t>
+          <t>Head of Engineering</t>
         </is>
       </c>
       <c r="L5" s="3" t="inlineStr">
@@ -980,7 +980,7 @@
       </c>
       <c r="K6" s="3" t="inlineStr">
         <is>
-          <t>Release mgr</t>
+          <t>Head of Engineering</t>
         </is>
       </c>
       <c r="L6" s="3" t="inlineStr">
@@ -1047,7 +1047,7 @@
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>Release mgr</t>
+          <t>Head of Engineering</t>
         </is>
       </c>
       <c r="L7" s="3" t="inlineStr">
@@ -1114,7 +1114,7 @@
       </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
-          <t>Release mgr</t>
+          <t>Head of Engineering</t>
         </is>
       </c>
       <c r="L8" s="3" t="inlineStr">
@@ -1248,7 +1248,7 @@
       </c>
       <c r="K10" s="3" t="inlineStr">
         <is>
-          <t>Release mgr</t>
+          <t>Head of Engineering</t>
         </is>
       </c>
       <c r="L10" s="3" t="inlineStr">
@@ -1315,7 +1315,7 @@
       </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
-          <t>Release mgr</t>
+          <t>Head of Engineering</t>
         </is>
       </c>
       <c r="L11" s="3" t="inlineStr">
@@ -1382,7 +1382,7 @@
       </c>
       <c r="K12" s="3" t="inlineStr">
         <is>
-          <t>Release mgr</t>
+          <t>Head of Engineering</t>
         </is>
       </c>
       <c r="L12" s="3" t="inlineStr">
@@ -1449,7 +1449,7 @@
       </c>
       <c r="K13" s="3" t="inlineStr">
         <is>
-          <t>Release mgr</t>
+          <t>Head of Engineering</t>
         </is>
       </c>
       <c r="L13" s="3" t="inlineStr">
@@ -1516,7 +1516,7 @@
       </c>
       <c r="K14" s="3" t="inlineStr">
         <is>
-          <t>Release mgr</t>
+          <t>Head of Engineering</t>
         </is>
       </c>
       <c r="L14" s="3" t="inlineStr">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="K15" s="3" t="inlineStr">
         <is>
-          <t>Release mgr</t>
+          <t>Head of Engineering</t>
         </is>
       </c>
       <c r="L15" s="3" t="inlineStr">
@@ -2910,7 +2910,7 @@
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>Release Manager</t>
+          <t>Head of Engineering</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
@@ -2947,7 +2947,7 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Release Manager</t>
+          <t>Head of Engineering</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
@@ -2984,7 +2984,7 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Release Manager</t>
+          <t>Head of Engineering</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -3021,7 +3021,7 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Release Manager</t>
+          <t>Head of Engineering</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
@@ -3058,7 +3058,7 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Release Manager</t>
+          <t>Head of Engineering</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
@@ -3095,7 +3095,7 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Release Manager</t>
+          <t>Head of Engineering</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
@@ -3132,7 +3132,7 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Release Manager</t>
+          <t>Head of Engineering</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">

</xml_diff>